<commit_message>
Excel bien puesto Tiempos duración números
</commit_message>
<xml_diff>
--- a/datosSesionesPruebaMedias.xlsx
+++ b/datosSesionesPruebaMedias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hlocal\C_TFG\Datos\Mision Colombia-20260209T150018Z-3-001\jsonToCsv_TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5651021-4444-4F33-89E3-47BFCB2921D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B1FC6B-4C10-4AFD-BFC7-710FB22D9234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1400,16 +1400,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>52387</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>386715</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>82867</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
+      <xdr:colOff>1259205</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>159067</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -1445,7 +1445,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6810375" y="9196387"/>
+              <a:off x="7945755" y="9409747"/>
               <a:ext cx="4720590" cy="2636520"/>
             </a:xfrm>
             <a:prstGeom prst="rect">

</xml_diff>